<commit_message>
Update Shout form submission test cases
</commit_message>
<xml_diff>
--- a/outputs/shout-test-cases/Shout Test Cases.xlsx
+++ b/outputs/shout-test-cases/Shout Test Cases.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Wordpress-Website" sheetId="1" r:id="R9f66ea0161ed4d96"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Wordpress-Website" sheetId="1" r:id="R721225279c614117"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -134,7 +134,95 @@
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
   </x:cellStyles>
-  <x:dxfs count="4">
+  <x:dxfs count="12">
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF137333"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFE6F4EA"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FFC5221F"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFFCE8E6"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FFB06000"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFFEF7E0"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FFC5221F"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFFCE8E6"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF137333"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFE6F4EA"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FFC5221F"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFFCE8E6"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FFB06000"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFFEF7E0"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FFC5221F"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFFCE8E6"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
     <x:dxf>
       <x:font>
         <x:b/>
@@ -184,8 +272,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="WPWebsiteTestCases" displayName="WPWebsiteTestCases" ref="A5:Q53" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A5:Q53"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="WPWebsiteTestCases" displayName="WPWebsiteTestCases" ref="A5:Q61" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A5:Q61"/>
   <x:tableColumns count="17">
     <x:tableColumn id="1" name="Case ID"/>
     <x:tableColumn id="2" name="Form"/>
@@ -582,9 +670,9 @@
       <x:c r="N6" s="16" t="str">
         <x:v>Not Run</x:v>
       </x:c>
-      <x:c r="O6" s="16" t="str"/>
-      <x:c r="P6" s="16" t="str"/>
-      <x:c r="Q6" s="16" t="str"/>
+      <x:c r="O6" s="16"/>
+      <x:c r="P6" s="16"/>
+      <x:c r="Q6" s="16"/>
     </x:row>
     <x:row r="7" ht="72" customHeight="1">
       <x:c r="A7" s="16" t="str">
@@ -629,9 +717,9 @@
       <x:c r="N7" s="16" t="str">
         <x:v>Not Run</x:v>
       </x:c>
-      <x:c r="O7" s="16" t="str"/>
-      <x:c r="P7" s="16" t="str"/>
-      <x:c r="Q7" s="16" t="str"/>
+      <x:c r="O7" s="16"/>
+      <x:c r="P7" s="16"/>
+      <x:c r="Q7" s="16"/>
     </x:row>
     <x:row r="8" ht="72" customHeight="1">
       <x:c r="A8" s="16" t="str">
@@ -676,8 +764,8 @@
       <x:c r="N8" s="16" t="str">
         <x:v>Not Run</x:v>
       </x:c>
-      <x:c r="O8" s="16" t="str"/>
-      <x:c r="P8" s="16" t="str"/>
+      <x:c r="O8" s="16"/>
+      <x:c r="P8" s="16"/>
       <x:c r="Q8" s="16" t="str">
         <x:v>Role comparison is case-insensitive after trimming.</x:v>
       </x:c>
@@ -725,9 +813,9 @@
       <x:c r="N9" s="16" t="str">
         <x:v>Not Run</x:v>
       </x:c>
-      <x:c r="O9" s="16" t="str"/>
-      <x:c r="P9" s="16" t="str"/>
-      <x:c r="Q9" s="16" t="str"/>
+      <x:c r="O9" s="16"/>
+      <x:c r="P9" s="16"/>
+      <x:c r="Q9" s="16"/>
     </x:row>
     <x:row r="10" ht="72" customHeight="1">
       <x:c r="A10" s="16" t="str">
@@ -772,9 +860,9 @@
       <x:c r="N10" s="16" t="str">
         <x:v>Not Run</x:v>
       </x:c>
-      <x:c r="O10" s="16" t="str"/>
-      <x:c r="P10" s="16" t="str"/>
-      <x:c r="Q10" s="16" t="str"/>
+      <x:c r="O10" s="16"/>
+      <x:c r="P10" s="16"/>
+      <x:c r="Q10" s="16"/>
     </x:row>
     <x:row r="11" ht="72" customHeight="1">
       <x:c r="A11" s="16" t="str">
@@ -819,9 +907,9 @@
       <x:c r="N11" s="16" t="str">
         <x:v>Not Run</x:v>
       </x:c>
-      <x:c r="O11" s="16" t="str"/>
-      <x:c r="P11" s="16" t="str"/>
-      <x:c r="Q11" s="16" t="str"/>
+      <x:c r="O11" s="16"/>
+      <x:c r="P11" s="16"/>
+      <x:c r="Q11" s="16"/>
     </x:row>
     <x:row r="12" ht="72" customHeight="1">
       <x:c r="A12" s="16" t="str">
@@ -866,9 +954,9 @@
       <x:c r="N12" s="16" t="str">
         <x:v>Not Run</x:v>
       </x:c>
-      <x:c r="O12" s="16" t="str"/>
-      <x:c r="P12" s="16" t="str"/>
-      <x:c r="Q12" s="16" t="str"/>
+      <x:c r="O12" s="16"/>
+      <x:c r="P12" s="16"/>
+      <x:c r="Q12" s="16"/>
     </x:row>
     <x:row r="13" ht="72" customHeight="1">
       <x:c r="A13" s="16" t="str">
@@ -913,9 +1001,9 @@
       <x:c r="N13" s="16" t="str">
         <x:v>Not Run</x:v>
       </x:c>
-      <x:c r="O13" s="16" t="str"/>
-      <x:c r="P13" s="16" t="str"/>
-      <x:c r="Q13" s="16" t="str"/>
+      <x:c r="O13" s="16"/>
+      <x:c r="P13" s="16"/>
+      <x:c r="Q13" s="16"/>
     </x:row>
     <x:row r="14" ht="72" customHeight="1">
       <x:c r="A14" s="16" t="str">
@@ -960,9 +1048,9 @@
       <x:c r="N14" s="16" t="str">
         <x:v>Not Run</x:v>
       </x:c>
-      <x:c r="O14" s="16" t="str"/>
-      <x:c r="P14" s="16" t="str"/>
-      <x:c r="Q14" s="16" t="str"/>
+      <x:c r="O14" s="16"/>
+      <x:c r="P14" s="16"/>
+      <x:c r="Q14" s="16"/>
     </x:row>
     <x:row r="15" ht="72" customHeight="1">
       <x:c r="A15" s="16" t="str">
@@ -1007,9 +1095,9 @@
       <x:c r="N15" s="16" t="str">
         <x:v>Not Run</x:v>
       </x:c>
-      <x:c r="O15" s="16" t="str"/>
-      <x:c r="P15" s="16" t="str"/>
-      <x:c r="Q15" s="16" t="str"/>
+      <x:c r="O15" s="16"/>
+      <x:c r="P15" s="16"/>
+      <x:c r="Q15" s="16"/>
     </x:row>
     <x:row r="16" ht="72" customHeight="1">
       <x:c r="A16" s="16" t="str">
@@ -1054,9 +1142,9 @@
       <x:c r="N16" s="16" t="str">
         <x:v>Not Run</x:v>
       </x:c>
-      <x:c r="O16" s="16" t="str"/>
-      <x:c r="P16" s="16" t="str"/>
-      <x:c r="Q16" s="16" t="str"/>
+      <x:c r="O16" s="16"/>
+      <x:c r="P16" s="16"/>
+      <x:c r="Q16" s="16"/>
     </x:row>
     <x:row r="17" ht="72" customHeight="1">
       <x:c r="A17" s="16" t="str">
@@ -1101,9 +1189,9 @@
       <x:c r="N17" s="16" t="str">
         <x:v>Not Run</x:v>
       </x:c>
-      <x:c r="O17" s="16" t="str"/>
-      <x:c r="P17" s="16" t="str"/>
-      <x:c r="Q17" s="16" t="str"/>
+      <x:c r="O17" s="16"/>
+      <x:c r="P17" s="16"/>
+      <x:c r="Q17" s="16"/>
     </x:row>
     <x:row r="18" ht="72" customHeight="1">
       <x:c r="A18" s="16" t="str">
@@ -1148,9 +1236,9 @@
       <x:c r="N18" s="16" t="str">
         <x:v>Not Run</x:v>
       </x:c>
-      <x:c r="O18" s="16" t="str"/>
-      <x:c r="P18" s="16" t="str"/>
-      <x:c r="Q18" s="16" t="str"/>
+      <x:c r="O18" s="16"/>
+      <x:c r="P18" s="16"/>
+      <x:c r="Q18" s="16"/>
     </x:row>
     <x:row r="19" ht="72" customHeight="1">
       <x:c r="A19" s="16" t="str">
@@ -1195,9 +1283,9 @@
       <x:c r="N19" s="16" t="str">
         <x:v>Not Run</x:v>
       </x:c>
-      <x:c r="O19" s="16" t="str"/>
-      <x:c r="P19" s="16" t="str"/>
-      <x:c r="Q19" s="16" t="str"/>
+      <x:c r="O19" s="16"/>
+      <x:c r="P19" s="16"/>
+      <x:c r="Q19" s="16"/>
     </x:row>
     <x:row r="20" ht="72" customHeight="1">
       <x:c r="A20" s="16" t="str">
@@ -1242,8 +1330,8 @@
       <x:c r="N20" s="16" t="str">
         <x:v>Not Run</x:v>
       </x:c>
-      <x:c r="O20" s="16" t="str"/>
-      <x:c r="P20" s="16" t="str"/>
+      <x:c r="O20" s="16"/>
+      <x:c r="P20" s="16"/>
       <x:c r="Q20" s="16" t="str">
         <x:v>Expected contact deduplication ultimately depends on GHL upsert behavior.</x:v>
       </x:c>
@@ -1265,7 +1353,7 @@
         <x:v>Positive</x:v>
       </x:c>
       <x:c r="F21" s="16" t="str">
-        <x:v>Valid QA contact/opportunity IDs; GHL configured; relevant opportunity custom fields exist.</x:v>
+        <x:v>Valid QA contact/opportunity IDs; GHL configured; relevant Contact product fields and retained Opportunity fields exist.</x:v>
       </x:c>
       <x:c r="G21" s="16" t="str">
         <x:v>Populate one or more text/select fields across the allowed event sections; no file upload.</x:v>
@@ -1277,23 +1365,23 @@
         <x:v>HTTP success with success=true, 'Event details were submitted.', and the mapped updated_fields list.</x:v>
       </x:c>
       <x:c r="J21" s="16" t="str">
-        <x:v>Contact gets strong lead; lead tag is removed. Failures of either tag operation are non-blocking.</x:v>
+        <x:v>Mapped non-empty product fields are updated on the Contact; strong lead is added and lead is removed only after all GHL field writes succeed.</x:v>
       </x:c>
       <x:c r="K21" s="16" t="str">
-        <x:v>Mapped non-empty opportunity custom fields are updated.</x:v>
+        <x:v>Only submitted retained fields (opportunity.item_finish, opportunity.item_type, and opportunity.venue_size) are updated.</x:v>
       </x:c>
       <x:c r="L21" s="16" t="str">
-        <x:v>Progressive webhook is sent after the opportunity update; success is logged.</x:v>
+        <x:v>The unchanged progressive webhook is sent after the Contact and Opportunity updates; success is logged.</x:v>
       </x:c>
       <x:c r="M21" s="16" t="str">
-        <x:v>No appointment is created and no WordPress file is uploaded.</x:v>
+        <x:v>No product-specific Opportunity custom field, appointment, or WordPress file is created.</x:v>
       </x:c>
       <x:c r="N21" s="16" t="str">
         <x:v>Not Run</x:v>
       </x:c>
-      <x:c r="O21" s="16" t="str"/>
-      <x:c r="P21" s="16" t="str"/>
-      <x:c r="Q21" s="16" t="str"/>
+      <x:c r="O21" s="16"/>
+      <x:c r="P21" s="16"/>
+      <x:c r="Q21" s="16"/>
     </x:row>
     <x:row r="22" ht="72" customHeight="1">
       <x:c r="A22" s="16" t="str">
@@ -1303,7 +1391,7 @@
         <x:v>Progressive Form (HTML/REST)</x:v>
       </x:c>
       <x:c r="C22" s="16" t="str">
-        <x:v>All supported standard fields are mapped correctly</x:v>
+        <x:v>All supported non-file fields map to the correct Contact and Opportunity destinations</x:v>
       </x:c>
       <x:c r="D22" s="16" t="str">
         <x:v>P1</x:v>
@@ -1312,35 +1400,35 @@
         <x:v>Positive</x:v>
       </x:c>
       <x:c r="F22" s="16" t="str">
-        <x:v>All progressive opportunity custom-field keys exist in GHL.</x:v>
+        <x:v>All progressive HTML/REST Contact product fields and the three retained Opportunity custom fields exist in GHL.</x:v>
       </x:c>
       <x:c r="G22" s="16" t="str">
-        <x:v>Populate representative values for quantities, sizes/types, inspiration URL/text fields, notes, finish, item type, and venue size.</x:v>
+        <x:v>Populate quantities, sizes/types, notes, dance-floor finish/type, and venue size; do not attach files.</x:v>
       </x:c>
       <x:c r="H22" s="16" t="str">
         <x:v>Submit the Progressive Form once without files.</x:v>
       </x:c>
       <x:c r="I22" s="16" t="str">
-        <x:v>Success response lists every mapped custom-field key that was updated.</x:v>
+        <x:v>Success response lists the mapped contact.* keys and the three submitted opportunity.* keys.</x:v>
       </x:c>
       <x:c r="J22" s="16" t="str">
-        <x:v>Strong lead is added and lead is removed.</x:v>
+        <x:v>Each non-empty product field lands in its exact Contact custom field; blank product fields are omitted and existing values remain unchanged.</x:v>
       </x:c>
       <x:c r="K22" s="16" t="str">
-        <x:v>Each non-empty form field lands in its corresponding opportunity custom field; empty fields are omitted.</x:v>
+        <x:v>Only opportunity.item_finish, opportunity.item_type, and opportunity.venue_size are updated when submitted.</x:v>
       </x:c>
       <x:c r="L22" s="16" t="str">
-        <x:v>Webhook payload contains IDs, venue size, product type/floor, and the configured detail/notes fields.</x:v>
+        <x:v>Webhook payload remains unchanged: IDs, venue size, product type/finish, and configured size/notes fields.</x:v>
       </x:c>
       <x:c r="M22" s="16" t="str">
-        <x:v>No blank custom-field values overwrite fields that were not submitted.</x:v>
+        <x:v>Legacy product-specific Opportunity values are neither updated nor cleared.</x:v>
       </x:c>
       <x:c r="N22" s="16" t="str">
         <x:v>Not Run</x:v>
       </x:c>
-      <x:c r="O22" s="16" t="str"/>
-      <x:c r="P22" s="16" t="str"/>
-      <x:c r="Q22" s="16" t="str"/>
+      <x:c r="O22" s="16"/>
+      <x:c r="P22" s="16"/>
+      <x:c r="Q22" s="16"/>
     </x:row>
     <x:row r="23" ht="72" customHeight="1">
       <x:c r="A23" s="16" t="str">
@@ -1359,7 +1447,7 @@
         <x:v>Positive</x:v>
       </x:c>
       <x:c r="F23" s="16" t="str">
-        <x:v>Valid IDs; target file custom field exists; WordPress uploads are writable.</x:v>
+        <x:v>Valid IDs; target Contact File Upload custom field exists; WordPress uploads are writable.</x:v>
       </x:c>
       <x:c r="G23" s="16" t="str">
         <x:v>Valid JPG, PNG, GIF, PDF, DOC, DOCX, XLS, or CSV plus standard event details.</x:v>
@@ -1371,23 +1459,23 @@
         <x:v>HTTP success lists both standard and file custom-field keys.</x:v>
       </x:c>
       <x:c r="J23" s="16" t="str">
-        <x:v>Strong lead is added and lead is removed.</x:v>
+        <x:v>Standard Contact fields update first; the Contact inspiration field is cleared and then set to the new public WordPress upload URL.</x:v>
       </x:c>
       <x:c r="K23" s="16" t="str">
-        <x:v>Standard fields update first; target file field is cleared and then set to the new public WordPress upload URL.</x:v>
+        <x:v>Retained Opportunity fields update only after all Contact writes succeed.</x:v>
       </x:c>
       <x:c r="L23" s="16" t="str">
-        <x:v>File is stored in WordPress with a unique timestamp/random suffix; webhook is sent.</x:v>
+        <x:v>File is stored in WordPress with a unique timestamp/random suffix; webhook is sent after both destinations succeed.</x:v>
       </x:c>
       <x:c r="M23" s="16" t="str">
-        <x:v>No appointment is created.</x:v>
+        <x:v>No legacy product-specific Opportunity file field is updated.</x:v>
       </x:c>
       <x:c r="N23" s="16" t="str">
         <x:v>Not Run</x:v>
       </x:c>
-      <x:c r="O23" s="16" t="str"/>
-      <x:c r="P23" s="16" t="str"/>
-      <x:c r="Q23" s="16" t="str"/>
+      <x:c r="O23" s="16"/>
+      <x:c r="P23" s="16"/>
+      <x:c r="Q23" s="16"/>
     </x:row>
     <x:row r="24" ht="72" customHeight="1">
       <x:c r="A24" s="16" t="str">
@@ -1406,7 +1494,7 @@
         <x:v>Positive</x:v>
       </x:c>
       <x:c r="F24" s="16" t="str">
-        <x:v>Opportunity already has a file value in the target custom field.</x:v>
+        <x:v>Contact already has a file value in the target inspiration custom field.</x:v>
       </x:c>
       <x:c r="G24" s="16" t="str">
         <x:v>Upload a different valid file to the same field.</x:v>
@@ -1418,10 +1506,10 @@
         <x:v>Submission succeeds.</x:v>
       </x:c>
       <x:c r="J24" s="16" t="str">
-        <x:v>Strong lead/lead tag operations run.</x:v>
+        <x:v>Existing Contact file-field value is cleared, then replaced with the new upload URL.</x:v>
       </x:c>
       <x:c r="K24" s="16" t="str">
-        <x:v>Existing GHL file custom-field value is cleared, then replaced with the new upload URL.</x:v>
+        <x:v>Legacy Opportunity inspiration values remain unchanged.</x:v>
       </x:c>
       <x:c r="L24" s="16" t="str">
         <x:v>A new uniquely named WordPress file is created and webhook is sent.</x:v>
@@ -1432,9 +1520,9 @@
       <x:c r="N24" s="16" t="str">
         <x:v>Not Run</x:v>
       </x:c>
-      <x:c r="O24" s="16" t="str"/>
-      <x:c r="P24" s="16" t="str"/>
-      <x:c r="Q24" s="16" t="str"/>
+      <x:c r="O24" s="16"/>
+      <x:c r="P24" s="16"/>
+      <x:c r="Q24" s="16"/>
     </x:row>
     <x:row r="25" ht="72" customHeight="1">
       <x:c r="A25" s="16" t="str">
@@ -1456,7 +1544,7 @@
         <x:v>Valid contact/opportunity IDs; GHL configured.</x:v>
       </x:c>
       <x:c r="G25" s="16" t="str">
-        <x:v>Only IDs or fields that do not map to configured opportunity custom fields.</x:v>
+        <x:v>Only IDs or fields that do not map to configured Contact or retained Opportunity custom fields.</x:v>
       </x:c>
       <x:c r="H25" s="16" t="str">
         <x:v>Submit the Progressive Form once.</x:v>
@@ -1465,10 +1553,10 @@
         <x:v>HTTP success with 'No event details were submitted.' and updated_fields=[].</x:v>
       </x:c>
       <x:c r="J25" s="16" t="str">
-        <x:v>No tag add/remove calls occur on this code path.</x:v>
+        <x:v>No Contact custom-field or tag update occurs.</x:v>
       </x:c>
       <x:c r="K25" s="16" t="str">
-        <x:v>No opportunity update call occurs.</x:v>
+        <x:v>No Opportunity update occurs.</x:v>
       </x:c>
       <x:c r="L25" s="16" t="str">
         <x:v>Progressive webhook is still sent with IDs and available payload values.</x:v>
@@ -1479,9 +1567,9 @@
       <x:c r="N25" s="16" t="str">
         <x:v>Not Run</x:v>
       </x:c>
-      <x:c r="O25" s="16" t="str"/>
-      <x:c r="P25" s="16" t="str"/>
-      <x:c r="Q25" s="16" t="str"/>
+      <x:c r="O25" s="16"/>
+      <x:c r="P25" s="16"/>
+      <x:c r="Q25" s="16"/>
     </x:row>
     <x:row r="26" ht="72" customHeight="1">
       <x:c r="A26" s="16" t="str">
@@ -1512,10 +1600,10 @@
         <x:v>HTTP 400 error: 'Contact ID and opportunity ID are required.'</x:v>
       </x:c>
       <x:c r="J26" s="16" t="str">
-        <x:v>No tag changes occur.</x:v>
+        <x:v>No Contact custom-field or tag update occurs.</x:v>
       </x:c>
       <x:c r="K26" s="16" t="str">
-        <x:v>No opportunity update occurs.</x:v>
+        <x:v>No Opportunity update occurs.</x:v>
       </x:c>
       <x:c r="L26" s="16" t="str">
         <x:v>Missing-ID condition is logged.</x:v>
@@ -1526,9 +1614,9 @@
       <x:c r="N26" s="16" t="str">
         <x:v>Not Run</x:v>
       </x:c>
-      <x:c r="O26" s="16" t="str"/>
-      <x:c r="P26" s="16" t="str"/>
-      <x:c r="Q26" s="16" t="str"/>
+      <x:c r="O26" s="16"/>
+      <x:c r="P26" s="16"/>
+      <x:c r="Q26" s="16"/>
     </x:row>
     <x:row r="27" ht="72" customHeight="1">
       <x:c r="A27" s="16" t="str">
@@ -1559,10 +1647,10 @@
         <x:v>HTTP 400 missing-IDs error.</x:v>
       </x:c>
       <x:c r="J27" s="16" t="str">
-        <x:v>No tag changes occur.</x:v>
+        <x:v>No Contact custom-field or tag update occurs.</x:v>
       </x:c>
       <x:c r="K27" s="16" t="str">
-        <x:v>No opportunity update occurs.</x:v>
+        <x:v>No Opportunity update occurs.</x:v>
       </x:c>
       <x:c r="L27" s="16" t="str">
         <x:v>The file is uploaded before ID validation and may remain as an orphaned WordPress upload.</x:v>
@@ -1573,8 +1661,8 @@
       <x:c r="N27" s="16" t="str">
         <x:v>Not Run</x:v>
       </x:c>
-      <x:c r="O27" s="16" t="str"/>
-      <x:c r="P27" s="16" t="str"/>
+      <x:c r="O27" s="16"/>
+      <x:c r="P27" s="16"/>
       <x:c r="Q27" s="16" t="str">
         <x:v>Current implementation validates IDs after processing uploaded files.</x:v>
       </x:c>
@@ -1608,10 +1696,10 @@
         <x:v>HTTP 500 error: 'GHL integration is not configured.'</x:v>
       </x:c>
       <x:c r="J28" s="16" t="str">
-        <x:v>No tag changes occur.</x:v>
+        <x:v>No Contact custom-field or tag update occurs.</x:v>
       </x:c>
       <x:c r="K28" s="16" t="str">
-        <x:v>No opportunity update occurs.</x:v>
+        <x:v>No Opportunity update occurs.</x:v>
       </x:c>
       <x:c r="L28" s="16" t="str">
         <x:v>Configuration error is logged.</x:v>
@@ -1622,9 +1710,9 @@
       <x:c r="N28" s="16" t="str">
         <x:v>Not Run</x:v>
       </x:c>
-      <x:c r="O28" s="16" t="str"/>
-      <x:c r="P28" s="16" t="str"/>
-      <x:c r="Q28" s="16" t="str"/>
+      <x:c r="O28" s="16"/>
+      <x:c r="P28" s="16"/>
+      <x:c r="Q28" s="16"/>
     </x:row>
     <x:row r="29" ht="72" customHeight="1">
       <x:c r="A29" s="16" t="str">
@@ -1655,10 +1743,10 @@
         <x:v>HTTP 400 upload error.</x:v>
       </x:c>
       <x:c r="J29" s="16" t="str">
-        <x:v>No tag changes occur.</x:v>
+        <x:v>No Contact custom-field or tag update occurs.</x:v>
       </x:c>
       <x:c r="K29" s="16" t="str">
-        <x:v>No opportunity update occurs.</x:v>
+        <x:v>No Opportunity update occurs.</x:v>
       </x:c>
       <x:c r="L29" s="16" t="str">
         <x:v>Upload failure message is returned.</x:v>
@@ -1669,9 +1757,9 @@
       <x:c r="N29" s="16" t="str">
         <x:v>Not Run</x:v>
       </x:c>
-      <x:c r="O29" s="16" t="str"/>
-      <x:c r="P29" s="16" t="str"/>
-      <x:c r="Q29" s="16" t="str"/>
+      <x:c r="O29" s="16"/>
+      <x:c r="P29" s="16"/>
+      <x:c r="Q29" s="16"/>
     </x:row>
     <x:row r="30" ht="72" customHeight="1">
       <x:c r="A30" s="16" t="str">
@@ -1681,7 +1769,7 @@
         <x:v>Progressive Form (HTML/REST)</x:v>
       </x:c>
       <x:c r="C30" s="16" t="str">
-        <x:v>Standard opportunity update fails</x:v>
+        <x:v>Contact custom-field update fails</x:v>
       </x:c>
       <x:c r="D30" s="16" t="str">
         <x:v>P0</x:v>
@@ -1690,25 +1778,25 @@
         <x:v>Negative</x:v>
       </x:c>
       <x:c r="F30" s="16" t="str">
-        <x:v>Valid IDs; force the GHL opportunity update to fail.</x:v>
+        <x:v>Valid IDs; force the first GHL Contact custom-field update to fail.</x:v>
       </x:c>
       <x:c r="G30" s="16" t="str">
-        <x:v>Mapped standard event details; no files.</x:v>
+        <x:v>Mapped non-file product details.</x:v>
       </x:c>
       <x:c r="H30" s="16" t="str">
         <x:v>Submit the Progressive Form once.</x:v>
       </x:c>
       <x:c r="I30" s="16" t="str">
-        <x:v>HTTP 502 error: 'GHL opportunity could not be updated.'</x:v>
+        <x:v>HTTP 502 error: 'GHL contact could not be updated.'</x:v>
       </x:c>
       <x:c r="J30" s="16" t="str">
-        <x:v>No tag changes occur because update success is required first.</x:v>
+        <x:v>Contact product changes are not confirmed; no tag update occurs.</x:v>
       </x:c>
       <x:c r="K30" s="16" t="str">
-        <x:v>Opportunity changes are not confirmed.</x:v>
+        <x:v>Opportunity update is not attempted.</x:v>
       </x:c>
       <x:c r="L30" s="16" t="str">
-        <x:v>Failure is logged.</x:v>
+        <x:v>Contact failure is logged.</x:v>
       </x:c>
       <x:c r="M30" s="16" t="str">
         <x:v>No webhook or appointment occurs.</x:v>
@@ -1716,9 +1804,9 @@
       <x:c r="N30" s="16" t="str">
         <x:v>Not Run</x:v>
       </x:c>
-      <x:c r="O30" s="16" t="str"/>
-      <x:c r="P30" s="16" t="str"/>
-      <x:c r="Q30" s="16" t="str"/>
+      <x:c r="O30" s="16"/>
+      <x:c r="P30" s="16"/>
+      <x:c r="Q30" s="16"/>
     </x:row>
     <x:row r="31" ht="72" customHeight="1">
       <x:c r="A31" s="16" t="str">
@@ -1728,7 +1816,7 @@
         <x:v>Progressive Form (HTML/REST)</x:v>
       </x:c>
       <x:c r="C31" s="16" t="str">
-        <x:v>Standard fields save but file-field write fails</x:v>
+        <x:v>Standard Contact fields save but file replacement fails</x:v>
       </x:c>
       <x:c r="D31" s="16" t="str">
         <x:v>P0</x:v>
@@ -1737,7 +1825,7 @@
         <x:v>Partial Success</x:v>
       </x:c>
       <x:c r="F31" s="16" t="str">
-        <x:v>Submit both standard and file fields; standard GHL update succeeds; final file-field update fails.</x:v>
+        <x:v>Submit standard and file fields; standard Contact update and file clear succeed; final Contact file write fails.</x:v>
       </x:c>
       <x:c r="G31" s="16" t="str">
         <x:v>Valid IDs, standard details, and a valid file.</x:v>
@@ -1749,23 +1837,23 @@
         <x:v>HTTP 502 error.</x:v>
       </x:c>
       <x:c r="J31" s="16" t="str">
-        <x:v>No tag changes occur.</x:v>
+        <x:v>Standard Contact fields remain updated; the failed file field may remain cleared.</x:v>
       </x:c>
       <x:c r="K31" s="16" t="str">
-        <x:v>Standard custom fields remain updated; file field is not confirmed set and may have been cleared.</x:v>
+        <x:v>Opportunity update is not attempted.</x:v>
       </x:c>
       <x:c r="L31" s="16" t="str">
         <x:v>Uploaded WordPress file remains; failure is logged.</x:v>
       </x:c>
       <x:c r="M31" s="16" t="str">
-        <x:v>No webhook is sent and no rollback restores the prior standard or file values.</x:v>
+        <x:v>No tag changes, webhook, rollback, or appointment occurs.</x:v>
       </x:c>
       <x:c r="N31" s="16" t="str">
         <x:v>Not Run</x:v>
       </x:c>
-      <x:c r="O31" s="16" t="str"/>
-      <x:c r="P31" s="16" t="str"/>
-      <x:c r="Q31" s="16" t="str"/>
+      <x:c r="O31" s="16"/>
+      <x:c r="P31" s="16"/>
+      <x:c r="Q31" s="16"/>
     </x:row>
     <x:row r="32" ht="72" customHeight="1">
       <x:c r="A32" s="16" t="str">
@@ -1775,16 +1863,16 @@
         <x:v>Progressive Form (HTML/REST)</x:v>
       </x:c>
       <x:c r="C32" s="16" t="str">
-        <x:v>File-field clear fails but replacement write succeeds</x:v>
+        <x:v>Contact file-field clear fails</x:v>
       </x:c>
       <x:c r="D32" s="16" t="str">
-        <x:v>P1</x:v>
+        <x:v>P0</x:v>
       </x:c>
       <x:c r="E32" s="16" t="str">
         <x:v>Partial Success</x:v>
       </x:c>
       <x:c r="F32" s="16" t="str">
-        <x:v>Force only the intermediate GHL clear request to fail; allow final file write to succeed.</x:v>
+        <x:v>Standard Contact fields save; force the Contact file-field clear request to fail.</x:v>
       </x:c>
       <x:c r="G32" s="16" t="str">
         <x:v>Valid IDs and valid replacement file.</x:v>
@@ -1793,26 +1881,26 @@
         <x:v>Submit the Progressive Form once.</x:v>
       </x:c>
       <x:c r="I32" s="16" t="str">
-        <x:v>HTTP success.</x:v>
+        <x:v>HTTP 502 error: 'GHL contact could not be updated.'</x:v>
       </x:c>
       <x:c r="J32" s="16" t="str">
-        <x:v>Strong lead/lead tag operations run.</x:v>
+        <x:v>Standard Contact fields remain updated; existing inspiration value may remain; replacement is not attempted.</x:v>
       </x:c>
       <x:c r="K32" s="16" t="str">
-        <x:v>Final file value is set despite the logged clear failure.</x:v>
+        <x:v>Opportunity update is not attempted.</x:v>
       </x:c>
       <x:c r="L32" s="16" t="str">
-        <x:v>WordPress file is uploaded; webhook is sent; clear failure is logged.</x:v>
+        <x:v>Uploaded WordPress file remains and the clear failure is logged.</x:v>
       </x:c>
       <x:c r="M32" s="16" t="str">
-        <x:v>The clear failure does not fail the submission.</x:v>
+        <x:v>No tag changes, webhook, rollback, or appointment occurs.</x:v>
       </x:c>
       <x:c r="N32" s="16" t="str">
         <x:v>Not Run</x:v>
       </x:c>
-      <x:c r="O32" s="16" t="str"/>
-      <x:c r="P32" s="16" t="str"/>
-      <x:c r="Q32" s="16" t="str"/>
+      <x:c r="O32" s="16"/>
+      <x:c r="P32" s="16"/>
+      <x:c r="Q32" s="16"/>
     </x:row>
     <x:row r="33" ht="72" customHeight="1">
       <x:c r="A33" s="16" t="str">
@@ -1831,7 +1919,7 @@
         <x:v>Partial Success</x:v>
       </x:c>
       <x:c r="F33" s="16" t="str">
-        <x:v>Opportunity update succeeds; force add-tag call to fail.</x:v>
+        <x:v>Contact and retained Opportunity updates succeed; force add-tag call to fail.</x:v>
       </x:c>
       <x:c r="G33" s="16" t="str">
         <x:v>Valid IDs and mapped details.</x:v>
@@ -1843,23 +1931,23 @@
         <x:v>HTTP success.</x:v>
       </x:c>
       <x:c r="J33" s="16" t="str">
-        <x:v>Strong lead may be absent; removal of lead is still attempted.</x:v>
+        <x:v>Product fields remain updated; strong lead may be absent; removal of lead is still attempted.</x:v>
       </x:c>
       <x:c r="K33" s="16" t="str">
-        <x:v>Opportunity fields remain updated.</x:v>
+        <x:v>Retained Opportunity fields remain updated.</x:v>
       </x:c>
       <x:c r="L33" s="16" t="str">
         <x:v>Tag failure is logged; webhook is still sent.</x:v>
       </x:c>
       <x:c r="M33" s="16" t="str">
-        <x:v>Opportunity update is not rolled back.</x:v>
+        <x:v>Successful Contact and Opportunity updates are not rolled back.</x:v>
       </x:c>
       <x:c r="N33" s="16" t="str">
         <x:v>Not Run</x:v>
       </x:c>
-      <x:c r="O33" s="16" t="str"/>
-      <x:c r="P33" s="16" t="str"/>
-      <x:c r="Q33" s="16" t="str"/>
+      <x:c r="O33" s="16"/>
+      <x:c r="P33" s="16"/>
+      <x:c r="Q33" s="16"/>
     </x:row>
     <x:row r="34" ht="72" customHeight="1">
       <x:c r="A34" s="16" t="str">
@@ -1878,7 +1966,7 @@
         <x:v>Partial Success</x:v>
       </x:c>
       <x:c r="F34" s="16" t="str">
-        <x:v>Opportunity update and add-tag succeed; force remove-tag call to fail.</x:v>
+        <x:v>Contact and retained Opportunity updates and add-tag succeed; force remove-tag call to fail.</x:v>
       </x:c>
       <x:c r="G34" s="16" t="str">
         <x:v>Valid IDs and mapped details.</x:v>
@@ -1890,23 +1978,23 @@
         <x:v>HTTP success.</x:v>
       </x:c>
       <x:c r="J34" s="16" t="str">
-        <x:v>Strong lead is added; lead may remain.</x:v>
+        <x:v>Product fields remain updated; strong lead is added; lead may remain.</x:v>
       </x:c>
       <x:c r="K34" s="16" t="str">
-        <x:v>Opportunity fields remain updated.</x:v>
+        <x:v>Retained Opportunity fields remain updated.</x:v>
       </x:c>
       <x:c r="L34" s="16" t="str">
         <x:v>Tag failure is logged; webhook is still sent.</x:v>
       </x:c>
       <x:c r="M34" s="16" t="str">
-        <x:v>Opportunity update and successful strong-lead tag are not rolled back.</x:v>
+        <x:v>Successful field writes and the strong-lead tag are not rolled back.</x:v>
       </x:c>
       <x:c r="N34" s="16" t="str">
         <x:v>Not Run</x:v>
       </x:c>
-      <x:c r="O34" s="16" t="str"/>
-      <x:c r="P34" s="16" t="str"/>
-      <x:c r="Q34" s="16" t="str"/>
+      <x:c r="O34" s="16"/>
+      <x:c r="P34" s="16"/>
+      <x:c r="Q34" s="16"/>
     </x:row>
     <x:row r="35" ht="72" customHeight="1">
       <x:c r="A35" s="16" t="str">
@@ -1925,7 +2013,7 @@
         <x:v>Partial Success</x:v>
       </x:c>
       <x:c r="F35" s="16" t="str">
-        <x:v>Opportunity and tag calls succeed; force webhook network/WP_Error.</x:v>
+        <x:v>Contact, retained Opportunity, and tag calls succeed; force webhook network/WP_Error.</x:v>
       </x:c>
       <x:c r="G35" s="16" t="str">
         <x:v>Valid IDs and mapped details.</x:v>
@@ -1937,10 +2025,10 @@
         <x:v>HTTP success remains unchanged.</x:v>
       </x:c>
       <x:c r="J35" s="16" t="str">
-        <x:v>Strong lead/lead tag changes remain applied.</x:v>
+        <x:v>Contact product fields and tag changes remain applied.</x:v>
       </x:c>
       <x:c r="K35" s="16" t="str">
-        <x:v>Opportunity fields remain updated.</x:v>
+        <x:v>Retained Opportunity fields remain updated.</x:v>
       </x:c>
       <x:c r="L35" s="16" t="str">
         <x:v>Webhook error is logged.</x:v>
@@ -1951,9 +2039,9 @@
       <x:c r="N35" s="16" t="str">
         <x:v>Not Run</x:v>
       </x:c>
-      <x:c r="O35" s="16" t="str"/>
-      <x:c r="P35" s="16" t="str"/>
-      <x:c r="Q35" s="16" t="str"/>
+      <x:c r="O35" s="16"/>
+      <x:c r="P35" s="16"/>
+      <x:c r="Q35" s="16"/>
     </x:row>
     <x:row r="36" ht="72" customHeight="1">
       <x:c r="A36" s="16" t="str">
@@ -1972,7 +2060,7 @@
         <x:v>Partial Success</x:v>
       </x:c>
       <x:c r="F36" s="16" t="str">
-        <x:v>Opportunity and tag calls succeed; webhook returns a non-2xx status.</x:v>
+        <x:v>Contact, retained Opportunity, and tag calls succeed; webhook returns non-2xx.</x:v>
       </x:c>
       <x:c r="G36" s="16" t="str">
         <x:v>Valid IDs and mapped details.</x:v>
@@ -1984,10 +2072,10 @@
         <x:v>HTTP success remains unchanged.</x:v>
       </x:c>
       <x:c r="J36" s="16" t="str">
-        <x:v>Strong lead/lead tag changes remain applied.</x:v>
+        <x:v>Contact product fields and tag changes remain applied.</x:v>
       </x:c>
       <x:c r="K36" s="16" t="str">
-        <x:v>Opportunity fields remain updated.</x:v>
+        <x:v>Retained Opportunity fields remain updated.</x:v>
       </x:c>
       <x:c r="L36" s="16" t="str">
         <x:v>Webhook status is logged as an error.</x:v>
@@ -1998,9 +2086,9 @@
       <x:c r="N36" s="16" t="str">
         <x:v>Not Run</x:v>
       </x:c>
-      <x:c r="O36" s="16" t="str"/>
-      <x:c r="P36" s="16" t="str"/>
-      <x:c r="Q36" s="16" t="str"/>
+      <x:c r="O36" s="16"/>
+      <x:c r="P36" s="16"/>
+      <x:c r="Q36" s="16"/>
     </x:row>
     <x:row r="37" ht="72" customHeight="1">
       <x:c r="A37" s="16" t="str">
@@ -2019,7 +2107,7 @@
         <x:v>Resilience</x:v>
       </x:c>
       <x:c r="F37" s="16" t="str">
-        <x:v>Relevant opportunity custom-field definitions cannot be resolved.</x:v>
+        <x:v>Relevant Contact and retained Opportunity custom-field definitions cannot be resolved.</x:v>
       </x:c>
       <x:c r="G37" s="16" t="str">
         <x:v>Valid IDs and otherwise mapped form field names.</x:v>
@@ -2031,10 +2119,10 @@
         <x:v>HTTP success says no event details were submitted; updated_fields=[].</x:v>
       </x:c>
       <x:c r="J37" s="16" t="str">
-        <x:v>No tag operations occur.</x:v>
+        <x:v>No Contact field or tag update occurs.</x:v>
       </x:c>
       <x:c r="K37" s="16" t="str">
-        <x:v>No opportunity update occurs.</x:v>
+        <x:v>No Opportunity update occurs.</x:v>
       </x:c>
       <x:c r="L37" s="16" t="str">
         <x:v>Webhook is still sent.</x:v>
@@ -2045,9 +2133,9 @@
       <x:c r="N37" s="16" t="str">
         <x:v>Not Run</x:v>
       </x:c>
-      <x:c r="O37" s="16" t="str"/>
-      <x:c r="P37" s="16" t="str"/>
-      <x:c r="Q37" s="16" t="str"/>
+      <x:c r="O37" s="16"/>
+      <x:c r="P37" s="16"/>
+      <x:c r="Q37" s="16"/>
     </x:row>
     <x:row r="38" ht="72" customHeight="1">
       <x:c r="A38" s="16" t="str">
@@ -2078,10 +2166,10 @@
         <x:v>Second request also returns success.</x:v>
       </x:c>
       <x:c r="J38" s="16" t="str">
-        <x:v>Add strong lead and remove lead calls are repeated.</x:v>
+        <x:v>The same Contact product fields are written again; add/remove tag calls are repeated.</x:v>
       </x:c>
       <x:c r="K38" s="16" t="str">
-        <x:v>The same opportunity fields are written again.</x:v>
+        <x:v>The same retained Opportunity fields are written again when included.</x:v>
       </x:c>
       <x:c r="L38" s="16" t="str">
         <x:v>Webhook is sent again.</x:v>
@@ -2092,9 +2180,9 @@
       <x:c r="N38" s="16" t="str">
         <x:v>Not Run</x:v>
       </x:c>
-      <x:c r="O38" s="16" t="str"/>
-      <x:c r="P38" s="16" t="str"/>
-      <x:c r="Q38" s="16" t="str"/>
+      <x:c r="O38" s="16"/>
+      <x:c r="P38" s="16"/>
+      <x:c r="Q38" s="16"/>
     </x:row>
     <x:row r="39" ht="72" customHeight="1">
       <x:c r="A39" s="16" t="str">
@@ -2125,10 +2213,10 @@
         <x:v>Second request returns success.</x:v>
       </x:c>
       <x:c r="J39" s="16" t="str">
-        <x:v>Tag operations are repeated.</x:v>
+        <x:v>Contact file field is cleared and set again to a new unique upload URL; tag operations repeat.</x:v>
       </x:c>
       <x:c r="K39" s="16" t="str">
-        <x:v>File field is cleared and set again to a new unique upload URL.</x:v>
+        <x:v>No legacy product-specific Opportunity file field is updated.</x:v>
       </x:c>
       <x:c r="L39" s="16" t="str">
         <x:v>A second WordPress file is stored and webhook is sent again.</x:v>
@@ -2139,9 +2227,9 @@
       <x:c r="N39" s="16" t="str">
         <x:v>Not Run</x:v>
       </x:c>
-      <x:c r="O39" s="16" t="str"/>
-      <x:c r="P39" s="16" t="str"/>
-      <x:c r="Q39" s="16" t="str"/>
+      <x:c r="O39" s="16"/>
+      <x:c r="P39" s="16"/>
+      <x:c r="Q39" s="16"/>
     </x:row>
     <x:row r="40" ht="72" customHeight="1">
       <x:c r="A40" s="16" t="str">
@@ -2169,13 +2257,13 @@
         <x:v>Submit the multipart request once.</x:v>
       </x:c>
       <x:c r="I40" s="16" t="str">
-        <x:v>Request can succeed.</x:v>
+        <x:v>Request can succeed when the client bypasses the single-file HTML constraint.</x:v>
       </x:c>
       <x:c r="J40" s="16" t="str">
-        <x:v>Tag operations run after the opportunity update.</x:v>
+        <x:v>Only the first uploaded URL is placed in the Contact inspiration field; tags run after all field updates.</x:v>
       </x:c>
       <x:c r="K40" s="16" t="str">
-        <x:v>Only the first uploaded URL is placed in the GHL custom field.</x:v>
+        <x:v>No legacy product-specific Opportunity file field is updated.</x:v>
       </x:c>
       <x:c r="L40" s="16" t="str">
         <x:v>All accepted files may be stored in WordPress; webhook is sent.</x:v>
@@ -2186,9 +2274,9 @@
       <x:c r="N40" s="16" t="str">
         <x:v>Not Run</x:v>
       </x:c>
-      <x:c r="O40" s="16" t="str"/>
-      <x:c r="P40" s="16" t="str"/>
-      <x:c r="Q40" s="16" t="str"/>
+      <x:c r="O40" s="16"/>
+      <x:c r="P40" s="16"/>
+      <x:c r="Q40" s="16"/>
     </x:row>
     <x:row r="41" ht="72" customHeight="1">
       <x:c r="A41" s="16" t="str">
@@ -2233,9 +2321,9 @@
       <x:c r="N41" s="16" t="str">
         <x:v>Not Run</x:v>
       </x:c>
-      <x:c r="O41" s="16" t="str"/>
-      <x:c r="P41" s="16" t="str"/>
-      <x:c r="Q41" s="16" t="str"/>
+      <x:c r="O41" s="16"/>
+      <x:c r="P41" s="16"/>
+      <x:c r="Q41" s="16"/>
     </x:row>
     <x:row r="42" ht="72" customHeight="1">
       <x:c r="A42" s="16" t="str">
@@ -2280,8 +2368,8 @@
       <x:c r="N42" s="16" t="str">
         <x:v>Not Run</x:v>
       </x:c>
-      <x:c r="O42" s="16" t="str"/>
-      <x:c r="P42" s="16" t="str"/>
+      <x:c r="O42" s="16"/>
+      <x:c r="P42" s="16"/>
       <x:c r="Q42" s="16" t="str">
         <x:v>Record whether GHL itself imposes any additional server-side restriction.</x:v>
       </x:c>
@@ -2329,9 +2417,9 @@
       <x:c r="N43" s="16" t="str">
         <x:v>Not Run</x:v>
       </x:c>
-      <x:c r="O43" s="16" t="str"/>
-      <x:c r="P43" s="16" t="str"/>
-      <x:c r="Q43" s="16" t="str"/>
+      <x:c r="O43" s="16"/>
+      <x:c r="P43" s="16"/>
+      <x:c r="Q43" s="16"/>
     </x:row>
     <x:row r="44" ht="72" customHeight="1">
       <x:c r="A44" s="16" t="str">
@@ -2376,9 +2464,9 @@
       <x:c r="N44" s="16" t="str">
         <x:v>Not Run</x:v>
       </x:c>
-      <x:c r="O44" s="16" t="str"/>
-      <x:c r="P44" s="16" t="str"/>
-      <x:c r="Q44" s="16" t="str"/>
+      <x:c r="O44" s="16"/>
+      <x:c r="P44" s="16"/>
+      <x:c r="Q44" s="16"/>
     </x:row>
     <x:row r="45" ht="72" customHeight="1">
       <x:c r="A45" s="16" t="str">
@@ -2423,9 +2511,9 @@
       <x:c r="N45" s="16" t="str">
         <x:v>Not Run</x:v>
       </x:c>
-      <x:c r="O45" s="16" t="str"/>
-      <x:c r="P45" s="16" t="str"/>
-      <x:c r="Q45" s="16" t="str"/>
+      <x:c r="O45" s="16"/>
+      <x:c r="P45" s="16"/>
+      <x:c r="Q45" s="16"/>
     </x:row>
     <x:row r="46" ht="72" customHeight="1">
       <x:c r="A46" s="16" t="str">
@@ -2470,9 +2558,9 @@
       <x:c r="N46" s="16" t="str">
         <x:v>Not Run</x:v>
       </x:c>
-      <x:c r="O46" s="16" t="str"/>
-      <x:c r="P46" s="16" t="str"/>
-      <x:c r="Q46" s="16" t="str"/>
+      <x:c r="O46" s="16"/>
+      <x:c r="P46" s="16"/>
+      <x:c r="Q46" s="16"/>
     </x:row>
     <x:row r="47" ht="72" customHeight="1">
       <x:c r="A47" s="16" t="str">
@@ -2517,9 +2605,9 @@
       <x:c r="N47" s="16" t="str">
         <x:v>Not Run</x:v>
       </x:c>
-      <x:c r="O47" s="16" t="str"/>
-      <x:c r="P47" s="16" t="str"/>
-      <x:c r="Q47" s="16" t="str"/>
+      <x:c r="O47" s="16"/>
+      <x:c r="P47" s="16"/>
+      <x:c r="Q47" s="16"/>
     </x:row>
     <x:row r="48" ht="72" customHeight="1">
       <x:c r="A48" s="16" t="str">
@@ -2564,9 +2652,9 @@
       <x:c r="N48" s="16" t="str">
         <x:v>Not Run</x:v>
       </x:c>
-      <x:c r="O48" s="16" t="str"/>
-      <x:c r="P48" s="16" t="str"/>
-      <x:c r="Q48" s="16" t="str"/>
+      <x:c r="O48" s="16"/>
+      <x:c r="P48" s="16"/>
+      <x:c r="Q48" s="16"/>
     </x:row>
     <x:row r="49" ht="72" customHeight="1">
       <x:c r="A49" s="16" t="str">
@@ -2611,9 +2699,9 @@
       <x:c r="N49" s="16" t="str">
         <x:v>Not Run</x:v>
       </x:c>
-      <x:c r="O49" s="16" t="str"/>
-      <x:c r="P49" s="16" t="str"/>
-      <x:c r="Q49" s="16" t="str"/>
+      <x:c r="O49" s="16"/>
+      <x:c r="P49" s="16"/>
+      <x:c r="Q49" s="16"/>
     </x:row>
     <x:row r="50" ht="72" customHeight="1">
       <x:c r="A50" s="16" t="str">
@@ -2658,9 +2746,9 @@
       <x:c r="N50" s="16" t="str">
         <x:v>Not Run</x:v>
       </x:c>
-      <x:c r="O50" s="16" t="str"/>
-      <x:c r="P50" s="16" t="str"/>
-      <x:c r="Q50" s="16" t="str"/>
+      <x:c r="O50" s="16"/>
+      <x:c r="P50" s="16"/>
+      <x:c r="Q50" s="16"/>
     </x:row>
     <x:row r="51" ht="72" customHeight="1">
       <x:c r="A51" s="16" t="str">
@@ -2705,9 +2793,9 @@
       <x:c r="N51" s="16" t="str">
         <x:v>Not Run</x:v>
       </x:c>
-      <x:c r="O51" s="16" t="str"/>
-      <x:c r="P51" s="16" t="str"/>
-      <x:c r="Q51" s="16" t="str"/>
+      <x:c r="O51" s="16"/>
+      <x:c r="P51" s="16"/>
+      <x:c r="Q51" s="16"/>
     </x:row>
     <x:row r="52" ht="72" customHeight="1">
       <x:c r="A52" s="16" t="str">
@@ -2752,9 +2840,9 @@
       <x:c r="N52" s="16" t="str">
         <x:v>Not Run</x:v>
       </x:c>
-      <x:c r="O52" s="16" t="str"/>
-      <x:c r="P52" s="16" t="str"/>
-      <x:c r="Q52" s="16" t="str"/>
+      <x:c r="O52" s="16"/>
+      <x:c r="P52" s="16"/>
+      <x:c r="Q52" s="16"/>
     </x:row>
     <x:row r="53" ht="72" customHeight="1">
       <x:c r="A53" s="17" t="str">
@@ -2799,9 +2887,393 @@
       <x:c r="N53" s="17" t="str">
         <x:v>Not Run</x:v>
       </x:c>
-      <x:c r="O53" s="17" t="str"/>
-      <x:c r="P53" s="17" t="str"/>
-      <x:c r="Q53" s="17" t="str"/>
+      <x:c r="O53" s="17"/>
+      <x:c r="P53" s="17"/>
+      <x:c r="Q53" s="17"/>
+    </x:row>
+    <x:row r="54" ht="72" customHeight="1">
+      <x:c r="A54" t="str">
+        <x:v>WP-PRO-021</x:v>
+      </x:c>
+      <x:c r="B54" t="str">
+        <x:v>Progressive Form (HTML/REST)</x:v>
+      </x:c>
+      <x:c r="C54" t="str">
+        <x:v>Dance Floor Wraps map to exact Contact fields</x:v>
+      </x:c>
+      <x:c r="D54" t="str">
+        <x:v>P0</x:v>
+      </x:c>
+      <x:c r="E54" t="str">
+        <x:v>Positive</x:v>
+      </x:c>
+      <x:c r="F54" t="str">
+        <x:v>The five Dance Floor Wraps Contact fields exist, including both File Upload fields.</x:v>
+      </x:c>
+      <x:c r="G54" t="str">
+        <x:v>Quantity, size, two inspiration files, and notes.</x:v>
+      </x:c>
+      <x:c r="H54" t="str">
+        <x:v>Submit only the Dance Floor Wraps section.</x:v>
+      </x:c>
+      <x:c r="I54" t="str">
+        <x:v>HTTP success lists all five mapped contact.* keys.</x:v>
+      </x:c>
+      <x:c r="J54" t="str">
+        <x:v>Values land in contact.floor_wrap_quantity, contact.floor_wrap_size, contact.dance_floor_inspiration_1, contact.dance_floor_inspiration_2, and contact.floor_wrap_notes.</x:v>
+      </x:c>
+      <x:c r="K54" t="str">
+        <x:v>Legacy opportunity.floor_wrap_* fields remain unchanged.</x:v>
+      </x:c>
+      <x:c r="L54" t="str">
+        <x:v>Both files are uploaded; webhook payload remains unchanged.</x:v>
+      </x:c>
+      <x:c r="M54" t="str">
+        <x:v>No unrelated product fields are updated.</x:v>
+      </x:c>
+      <x:c r="N54" t="str">
+        <x:v>Not Run</x:v>
+      </x:c>
+      <x:c r="O54"/>
+      <x:c r="P54"/>
+      <x:c r="Q54"/>
+    </x:row>
+    <x:row r="55" ht="72" customHeight="1">
+      <x:c r="A55" t="str">
+        <x:v>WP-PRO-022</x:v>
+      </x:c>
+      <x:c r="B55" t="str">
+        <x:v>Progressive Form (HTML/REST)</x:v>
+      </x:c>
+      <x:c r="C55" t="str">
+        <x:v>Aisles map to exact Contact fields</x:v>
+      </x:c>
+      <x:c r="D55" t="str">
+        <x:v>P0</x:v>
+      </x:c>
+      <x:c r="E55" t="str">
+        <x:v>Positive</x:v>
+      </x:c>
+      <x:c r="F55" t="str">
+        <x:v>The five Aisles Contact fields exist, including both File Upload fields.</x:v>
+      </x:c>
+      <x:c r="G55" t="str">
+        <x:v>Quantity, size, two inspiration files, and notes.</x:v>
+      </x:c>
+      <x:c r="H55" t="str">
+        <x:v>Submit only the Aisles section.</x:v>
+      </x:c>
+      <x:c r="I55" t="str">
+        <x:v>HTTP success lists all five mapped contact.* keys.</x:v>
+      </x:c>
+      <x:c r="J55" t="str">
+        <x:v>Values land in contact.aisle_quantity, contact.aisle_size, contact.aisle_inspiration_1, contact.aisle_inspiration_2, and contact.aisle_notes.</x:v>
+      </x:c>
+      <x:c r="K55" t="str">
+        <x:v>Legacy opportunity.aisle_* fields remain unchanged.</x:v>
+      </x:c>
+      <x:c r="L55" t="str">
+        <x:v>Both files are uploaded; webhook payload remains unchanged.</x:v>
+      </x:c>
+      <x:c r="M55" t="str">
+        <x:v>No unrelated product fields are updated.</x:v>
+      </x:c>
+      <x:c r="N55" t="str">
+        <x:v>Not Run</x:v>
+      </x:c>
+      <x:c r="O55"/>
+      <x:c r="P55"/>
+      <x:c r="Q55"/>
+    </x:row>
+    <x:row r="56" ht="72" customHeight="1">
+      <x:c r="A56" t="str">
+        <x:v>WP-PRO-023</x:v>
+      </x:c>
+      <x:c r="B56" t="str">
+        <x:v>Progressive Form (HTML/REST)</x:v>
+      </x:c>
+      <x:c r="C56" t="str">
+        <x:v>Breathtaking Enhancements map to exact Contact fields</x:v>
+      </x:c>
+      <x:c r="D56" t="str">
+        <x:v>P0</x:v>
+      </x:c>
+      <x:c r="E56" t="str">
+        <x:v>Positive</x:v>
+      </x:c>
+      <x:c r="F56" t="str">
+        <x:v>The five Breathtaking Enhancements Contact fields exist, including both File Upload fields.</x:v>
+      </x:c>
+      <x:c r="G56" t="str">
+        <x:v>Quantity, size/type, two inspiration files, and notes.</x:v>
+      </x:c>
+      <x:c r="H56" t="str">
+        <x:v>Submit only the Breathtaking Enhancements section.</x:v>
+      </x:c>
+      <x:c r="I56" t="str">
+        <x:v>HTTP success lists all five mapped contact.* keys.</x:v>
+      </x:c>
+      <x:c r="J56" t="str">
+        <x:v>Values land in contact.breathtaking_enhancements_quantity, contact.breathtaking_enhancements_size, contact.breathtaking_enhancements_inspiration_1, contact.breathtaking_enhancements_inspiration_2, and contact.breathtaking_enhancement_note.</x:v>
+      </x:c>
+      <x:c r="K56" t="str">
+        <x:v>Legacy opportunity.breathtaking_enhancements_* fields remain unchanged.</x:v>
+      </x:c>
+      <x:c r="L56" t="str">
+        <x:v>Both files are uploaded; webhook payload remains unchanged.</x:v>
+      </x:c>
+      <x:c r="M56" t="str">
+        <x:v>No unrelated product fields are updated.</x:v>
+      </x:c>
+      <x:c r="N56" t="str">
+        <x:v>Not Run</x:v>
+      </x:c>
+      <x:c r="O56"/>
+      <x:c r="P56"/>
+      <x:c r="Q56" t="str">
+        <x:v>Verify the note key is singular: breathtaking_enhancement_note.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="57" ht="72" customHeight="1">
+      <x:c r="A57" t="str">
+        <x:v>WP-PRO-024</x:v>
+      </x:c>
+      <x:c r="B57" t="str">
+        <x:v>Progressive Form (HTML/REST)</x:v>
+      </x:c>
+      <x:c r="C57" t="str">
+        <x:v>Specialized Touches map to exact Contact fields</x:v>
+      </x:c>
+      <x:c r="D57" t="str">
+        <x:v>P0</x:v>
+      </x:c>
+      <x:c r="E57" t="str">
+        <x:v>Positive</x:v>
+      </x:c>
+      <x:c r="F57" t="str">
+        <x:v>The five Specialized Touches Contact fields exist, including both File Upload fields.</x:v>
+      </x:c>
+      <x:c r="G57" t="str">
+        <x:v>Quantity, size/details, two inspiration files, and notes.</x:v>
+      </x:c>
+      <x:c r="H57" t="str">
+        <x:v>Submit only the Specialized Touches section.</x:v>
+      </x:c>
+      <x:c r="I57" t="str">
+        <x:v>HTTP success lists all five mapped contact.* keys.</x:v>
+      </x:c>
+      <x:c r="J57" t="str">
+        <x:v>Values land in contact.specialized_touches_quantity, contact.specialized_touches_size, contact.specialized_touches_inspiration_1, contact.specialized_touches_inspiration_2, and contact.specialized_touches_note.</x:v>
+      </x:c>
+      <x:c r="K57" t="str">
+        <x:v>Legacy opportunity.specialized_touches_* fields remain unchanged.</x:v>
+      </x:c>
+      <x:c r="L57" t="str">
+        <x:v>Both files are uploaded; webhook payload remains unchanged.</x:v>
+      </x:c>
+      <x:c r="M57" t="str">
+        <x:v>No unrelated product fields are updated.</x:v>
+      </x:c>
+      <x:c r="N57" t="str">
+        <x:v>Not Run</x:v>
+      </x:c>
+      <x:c r="O57"/>
+      <x:c r="P57"/>
+      <x:c r="Q57" t="str">
+        <x:v>Verify the note key is singular: specialized_touches_note.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="58" ht="72" customHeight="1">
+      <x:c r="A58" t="str">
+        <x:v>WP-PRO-025</x:v>
+      </x:c>
+      <x:c r="B58" t="str">
+        <x:v>Progressive Form (HTML/REST)</x:v>
+      </x:c>
+      <x:c r="C58" t="str">
+        <x:v>Individualized Accents map to exact Contact fields</x:v>
+      </x:c>
+      <x:c r="D58" t="str">
+        <x:v>P0</x:v>
+      </x:c>
+      <x:c r="E58" t="str">
+        <x:v>Positive</x:v>
+      </x:c>
+      <x:c r="F58" t="str">
+        <x:v>The five Individualized Accents Contact fields exist, including both File Upload fields.</x:v>
+      </x:c>
+      <x:c r="G58" t="str">
+        <x:v>Quantity, size/details, two inspiration files, and notes.</x:v>
+      </x:c>
+      <x:c r="H58" t="str">
+        <x:v>Submit only the Individualized Accents section.</x:v>
+      </x:c>
+      <x:c r="I58" t="str">
+        <x:v>HTTP success lists all five mapped contact.* keys.</x:v>
+      </x:c>
+      <x:c r="J58" t="str">
+        <x:v>Values land in contact.individualized_accents_quantity, contact.individualized_accents_size, contact.individualized_accents_inspiration_1, contact.individualized_accents_inspiration_2, and contact.individualized_accents_note.</x:v>
+      </x:c>
+      <x:c r="K58" t="str">
+        <x:v>Legacy opportunity.individualized_accents_* fields remain unchanged.</x:v>
+      </x:c>
+      <x:c r="L58" t="str">
+        <x:v>Both files are uploaded; webhook payload remains unchanged.</x:v>
+      </x:c>
+      <x:c r="M58" t="str">
+        <x:v>No unrelated product fields are updated.</x:v>
+      </x:c>
+      <x:c r="N58" t="str">
+        <x:v>Not Run</x:v>
+      </x:c>
+      <x:c r="O58"/>
+      <x:c r="P58"/>
+      <x:c r="Q58" t="str">
+        <x:v>Verify the note key is singular: individualized_accents_note.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="59" ht="72" customHeight="1">
+      <x:c r="A59" t="str">
+        <x:v>WP-PRO-026</x:v>
+      </x:c>
+      <x:c r="B59" t="str">
+        <x:v>Progressive Form (HTML/REST)</x:v>
+      </x:c>
+      <x:c r="C59" t="str">
+        <x:v>Only three general fields remain on Opportunity</x:v>
+      </x:c>
+      <x:c r="D59" t="str">
+        <x:v>P0</x:v>
+      </x:c>
+      <x:c r="E59" t="str">
+        <x:v>Regression</x:v>
+      </x:c>
+      <x:c r="F59" t="str">
+        <x:v>Contact product fields and the three retained Opportunity fields exist; legacy Opportunity product fields contain known values.</x:v>
+      </x:c>
+      <x:c r="G59" t="str">
+        <x:v>Submit product details plus dance_floor_wrap_finish, dance_floor_wrap_type, and venue_room_size.</x:v>
+      </x:c>
+      <x:c r="H59" t="str">
+        <x:v>Submit the Progressive Form once.</x:v>
+      </x:c>
+      <x:c r="I59" t="str">
+        <x:v>HTTP success lists Contact product keys plus opportunity.item_finish, opportunity.item_type, and opportunity.venue_size.</x:v>
+      </x:c>
+      <x:c r="J59" t="str">
+        <x:v>Product details update on the Contact.</x:v>
+      </x:c>
+      <x:c r="K59" t="str">
+        <x:v>Only opportunity.item_finish, opportunity.item_type, and opportunity.venue_size update; legacy product-specific Opportunity values remain unchanged.</x:v>
+      </x:c>
+      <x:c r="L59" t="str">
+        <x:v>Webhook payload remains unchanged and is sent after both updates.</x:v>
+      </x:c>
+      <x:c r="M59" t="str">
+        <x:v>No legacy Opportunity product field is cleared or overwritten.</x:v>
+      </x:c>
+      <x:c r="N59" t="str">
+        <x:v>Not Run</x:v>
+      </x:c>
+      <x:c r="O59"/>
+      <x:c r="P59"/>
+      <x:c r="Q59"/>
+    </x:row>
+    <x:row r="60" ht="72" customHeight="1">
+      <x:c r="A60" t="str">
+        <x:v>WP-PRO-027</x:v>
+      </x:c>
+      <x:c r="B60" t="str">
+        <x:v>Progressive Form (HTML/REST)</x:v>
+      </x:c>
+      <x:c r="C60" t="str">
+        <x:v>Contact succeeds but retained Opportunity update fails</x:v>
+      </x:c>
+      <x:c r="D60" t="str">
+        <x:v>P0</x:v>
+      </x:c>
+      <x:c r="E60" t="str">
+        <x:v>Partial Success</x:v>
+      </x:c>
+      <x:c r="F60" t="str">
+        <x:v>Contact update succeeds; force the retained Opportunity update to fail.</x:v>
+      </x:c>
+      <x:c r="G60" t="str">
+        <x:v>Valid product details plus one retained Opportunity field.</x:v>
+      </x:c>
+      <x:c r="H60" t="str">
+        <x:v>Submit the Progressive Form once.</x:v>
+      </x:c>
+      <x:c r="I60" t="str">
+        <x:v>HTTP 502 error: 'GHL opportunity could not be updated.'</x:v>
+      </x:c>
+      <x:c r="J60" t="str">
+        <x:v>Contact product fields remain saved because Contact is updated first; no tag changes occur.</x:v>
+      </x:c>
+      <x:c r="K60" t="str">
+        <x:v>Retained Opportunity change is not confirmed.</x:v>
+      </x:c>
+      <x:c r="L60" t="str">
+        <x:v>Opportunity failure is logged.</x:v>
+      </x:c>
+      <x:c r="M60" t="str">
+        <x:v>No rollback, webhook, or appointment occurs.</x:v>
+      </x:c>
+      <x:c r="N60" t="str">
+        <x:v>Not Run</x:v>
+      </x:c>
+      <x:c r="O60"/>
+      <x:c r="P60"/>
+      <x:c r="Q60" t="str">
+        <x:v>Retry is safe but repeats the Contact write.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="61" ht="72" customHeight="1">
+      <x:c r="A61" t="str">
+        <x:v>WP-PRO-028</x:v>
+      </x:c>
+      <x:c r="B61" t="str">
+        <x:v>Progressive Form (HTML/REST)</x:v>
+      </x:c>
+      <x:c r="C61" t="str">
+        <x:v>Blank product fields preserve existing Contact values</x:v>
+      </x:c>
+      <x:c r="D61" t="str">
+        <x:v>P0</x:v>
+      </x:c>
+      <x:c r="E61" t="str">
+        <x:v>Regression</x:v>
+      </x:c>
+      <x:c r="F61" t="str">
+        <x:v>Contact has existing values in product fields; at least one other mapped field will be submitted non-empty.</x:v>
+      </x:c>
+      <x:c r="G61" t="str">
+        <x:v>Leave one visible or hidden product field blank; populate another mapped product field.</x:v>
+      </x:c>
+      <x:c r="H61" t="str">
+        <x:v>Submit the Progressive Form once.</x:v>
+      </x:c>
+      <x:c r="I61" t="str">
+        <x:v>HTTP success lists only the non-empty mapped field.</x:v>
+      </x:c>
+      <x:c r="J61" t="str">
+        <x:v>Blank product field is omitted and its existing Contact value remains; the non-empty field updates normally.</x:v>
+      </x:c>
+      <x:c r="K61" t="str">
+        <x:v>No legacy product-specific Opportunity field is changed.</x:v>
+      </x:c>
+      <x:c r="L61" t="str">
+        <x:v>Tags and webhook run after successful mapped updates.</x:v>
+      </x:c>
+      <x:c r="M61" t="str">
+        <x:v>No blank value clears stored Contact data.</x:v>
+      </x:c>
+      <x:c r="N61" t="str">
+        <x:v>Not Run</x:v>
+      </x:c>
+      <x:c r="O61"/>
+      <x:c r="P61"/>
+      <x:c r="Q61"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -2817,7 +3289,15 @@
   <x:conditionalFormatting sqref="D6:D53">
     <x:cfRule type="containsText" dxfId="3" priority="4" operator="containsText" text="P0"/>
   </x:conditionalFormatting>
-  <x:dataValidations count="4">
+  <x:conditionalFormatting sqref="N6:N61">
+    <x:cfRule type="containsText" dxfId="8" priority="9" operator="containsText" text="Pass"/>
+    <x:cfRule type="containsText" dxfId="9" priority="10" operator="containsText" text="Fail"/>
+    <x:cfRule type="containsText" dxfId="10" priority="11" operator="containsText" text="Blocked"/>
+  </x:conditionalFormatting>
+  <x:conditionalFormatting sqref="D6:D61">
+    <x:cfRule type="containsText" dxfId="11" priority="12" operator="containsText" text="P0"/>
+  </x:conditionalFormatting>
+  <x:dataValidations count="8">
     <x:dataValidation type="list" sqref="B6:B53">
       <x:formula1>"Initial Form,Progressive Form (HTML/REST),Schedule Appointment Form"</x:formula1>
     </x:dataValidation>
@@ -2830,10 +3310,22 @@
     <x:dataValidation type="list" sqref="N6:N53">
       <x:formula1>"Not Run,Pass,Fail,Blocked,Not Applicable"</x:formula1>
     </x:dataValidation>
+    <x:dataValidation type="list" sqref="B6:B61">
+      <x:formula1>"Initial Form,Progressive Form (HTML/REST),Schedule Appointment Form"</x:formula1>
+    </x:dataValidation>
+    <x:dataValidation type="list" sqref="D6:D61">
+      <x:formula1>"P0,P1,P2"</x:formula1>
+    </x:dataValidation>
+    <x:dataValidation type="list" sqref="E6:E61">
+      <x:formula1>"Positive,Negative,Partial Success,Resilience,Duplicate Submission,Risk,Regression"</x:formula1>
+    </x:dataValidation>
+    <x:dataValidation type="list" sqref="N6:N61">
+      <x:formula1>"Not Run,Pass,Fail,Blocked,Not Applicable"</x:formula1>
+    </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd6c9a54c43e74f91"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9db4ba87bc5b4cdc"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>